<commit_message>
seperating transformer and bm25
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,71 @@
         <v>0.4760306064989383</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>(&lt;pyterrier._ops.SetUnion object at 0x000001F8DE300640&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000001F8DE92E350&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DE300770&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F88CBA35C0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DC933BF0&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001F8E006B4D0&gt;)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.2390363161097517</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.40578887498606</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>(&lt;pyterrier._ops.SetUnion object at 0x000001F8DE300640&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000001F8DE92E350&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DE300770&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F88CBA35C0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DC933BF0&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001F8E006B4D0&gt; &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.2333535064718376</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.4018028017422748</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>(&lt;pyterrier._ops.SetUnion object at 0x000001D056F00830&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000001D056F00D70&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001D056F00980&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001D056FCA850&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001D056FCA990&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001D056F00EC0&gt; &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.2512160736640014</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.4468742331918501</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.2337590751383574</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.3984588085424314</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TerrierRetr(BM25)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.2633463720353254</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.3981883051158283</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
adding saving the model test transfer
</commit_message>
<xml_diff>
--- a/evaluation_results.xlsx
+++ b/evaluation_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,136 +444,669 @@
           <t>ndcg_cut_10</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>xgboost_features</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Trans_model</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>(TerrierRetr(BM25) &gt;&gt; (TerrierRetr(Tf) ** TerrierRetr(PL2) ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x00000223DF084F50&gt;)</t>
+          <t>TerrierRetr(BM25)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2640165322538667</v>
+        <v>0.2633463720353254</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4288923247476766</v>
+        <v>0.3981883051158283</v>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>BM25 baseline robust 2004</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>(TerrierRetr(BM25) &gt;&gt; (TerrierRetr(Tf) ** TerrierRetr(PL2) ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x00000223F183C7D0&gt;)</t>
+          <t>(&lt;pyterrier._ops.SetUnion object at 0x00000171C65746E0&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x00000171C6574C20&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C6574830&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C666E0D0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C666E210&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x00000171C6574D70&gt; &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.2636832138379338</v>
+        <v>0.2299675215645097</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4328666394185419</v>
+        <v>0.3958134305111119</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>['bm25', 'TF', 'PL2', 'term_unique', 'term_full', 'term_first200', 'doc_length', 'query_length', 'ratio', 'first_match']</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>minilm</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>top 100 bm25+ Xgboost + minilm</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>(TerrierRetr(BM25) &gt;&gt; (TerrierRetr(Tf) ** TerrierRetr(PL2) ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001A33AE4CAD0&gt;)</t>
+          <t>(&lt;pyterrier._ops.SetUnion object at 0x00000171C65746E0&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x00000171C6574C20&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C6574830&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C666E0D0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C666E210&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x00000171C6574D70&gt; &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2636832138379338</v>
+        <v>0.2512160736640014</v>
       </c>
       <c r="C4" t="n">
-        <v>0.4328666394185419</v>
+        <v>0.4468742331918501</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>['bm25', 'TF', 'PL2', 'term_unique', 'term_full', 'term_first200', 'doc_length', 'query_length', 'ratio', 'first_match']</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>mpnet</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>top 100 bm25+ Xgboost + mpnet</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>(&lt;pyterrier._ops.SetUnion object at 0x000001949B4976F0&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x00000194A6A5FC50&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001949B4975C0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001949B496EA0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000019496D74A70&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x00000194A6A5F110&gt;)</t>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.09141840205407331</v>
+        <v>0.2337590751383574</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3209493560511296</v>
+        <v>0.3984588085424314</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>minilm</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>top 100 bm25 + minilm</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.2511027625386617</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.44281902353639</v>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>mpnet</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>top 100 bm25 + mpnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">top 100 bm25 + Xgboost </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">top 100 bm25 + Xgboost </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>top 100 bm25 + Xgboost -3 worst features</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>top 100 bm25 + Xgboost -3 worst features</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>(&lt;pyterrier._ops.SetUnion object at 0x0000019251400050&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x00000192514B97F0&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x00000192514B9550&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000019251400190&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000192514002D0&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x00000192514B9A90&gt;)</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B12" t="n">
         <v>0.2743828363576117</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C12" t="n">
         <v>0.4760306064989383</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>(&lt;pyterrier._ops.SetUnion object at 0x000001F8DE300640&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000001F8DE92E350&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DE300770&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F88CBA35C0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DC933BF0&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001F8E006B4D0&gt;)</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>0.2390363161097517</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.40578887498606</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>(&lt;pyterrier._ops.SetUnion object at 0x000001F8DE300640&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000001F8DE92E350&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DE300770&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F88CBA35C0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001F8DC933BF0&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001F8E006B4D0&gt; &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>0.2333535064718376</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.4018028017422748</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>(&lt;pyterrier._ops.SetUnion object at 0x000001D056F00830&gt; &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000001D056F00D70&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001D056F00980&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001D056FCA850&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001D056FCA990&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001D056F00EC0&gt; &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>0.2512160736640014</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.4468742331918501</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>bm25+ Xgboost(with trans)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" t="inlineStr"/>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run OWI BM25  </t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run OWI With ltr model </t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>top 100(bm25+pl2)+Xgboost + minilm -OWI</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>top 100(bm25+pl2)+Xgboost + mpnet -OWI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>top 100 bm25+ minilm -OWI</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>top 100 bm25+ mpnet -OWI</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TerrierRetr(BM25)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.2633463720353254</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0.3981883051158283</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>minilm</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TerrierRetr(BM25)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.2633463720353254</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0.3981883051158283</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>minilm</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x00000171C666CE10&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C626B570&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171C626BDF0&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000171D518B950&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x00000171C645DF30&gt;)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.2296936788139386</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0.4172254552213399</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>['bm25', 'TF', 'PL2', 'term_unique', 'term_full', 'term_first200', 'doc_length', 'query_length', 'ratio', 'first_match']</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>minilm</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(500) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000002C76B2C6F90&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000002C76B2C5940&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002C76B410550&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002C76B410690&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000002C76B2C7230&gt;)</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.2615874745068187</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0.4326216557552278</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000002D9DF286F90&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF285940&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC550&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC690&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000002D9ED9FCB90&gt;)</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.2296936788139386</v>
+      </c>
+      <c r="C28" t="n">
+        <v>0.4172254552213399</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000002D9DF286F90&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF285940&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC550&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC690&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000002D9ED9FCB90&gt; &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.2337590751383574</v>
+      </c>
+      <c r="C29" t="n">
+        <v>0.3984588085424314</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000002D9DF286F90&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF285940&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC550&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC690&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000002D9ED9FCB90&gt; &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.2511027625386617</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0.44281902353639</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B31" t="n">
+        <v>0.2511027625386617</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0.44281902353639</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
         <v>0.2337590751383574</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C32" t="n">
         <v>0.3984588085424314</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>TerrierRetr(BM25)</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>0.2633463720353254</v>
-      </c>
-      <c r="C11" t="n">
-        <v>0.3981883051158283</v>
-      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000002D9DF286F90&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF285940&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC550&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF3BC690&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000002D9ED9FCB90&gt; &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.2337590751383574</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0.3984588085424314</v>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.2337590751383574</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0.3984588085424314</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000002D9DF0D7C50&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF255F30&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF255480&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000002D9DF1D7530&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000002D9DF2542B0&gt;)</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.2612812405432577</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0.4786019597167245</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x0000017F59074190&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F58E11260&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F58C73A50&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x0000017F677B0B90&gt; &gt;&gt; pt.apply.doc_score() &gt;&gt; pt.apply.generic())</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.2337590751383574</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0.3984588085424314</v>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x0000017F59074190&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F58E11260&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F58C73A50&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x0000017F677B0B90&gt; &gt;&gt; pt.apply.doc_score() &gt;&gt; pt.apply.generic())</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.2337590751383574</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0.3984588085424314</v>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x0000017F59074190&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F58E11260&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F58C73A50&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x0000017F677B0B90&gt;)</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.2253728782255855</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0.416002551038688</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x0000017F7F828E10&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F5A600500&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000017F64E33230&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x0000017F590D5940&gt;)</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.223508759503423</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0.4055733978836211</v>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(500) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x000001B46B67AF90&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x000001B46B679940&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001B46B7B8550&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x000001B46B7B8690&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000001B46B67B230&gt; &gt;&gt; RankCutoff(100) &gt;&gt; pt.apply.doc_score())</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.2556362493640345</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0.466621809953758</v>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(500) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x0000025146AF1590&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x0000025146986650&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x00000250C26B5D90&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x000002508095F110&gt;)</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.2599895734934839</v>
+      </c>
+      <c r="C41" t="n">
+        <v>0.4186892318549046</v>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x0000025080C04910&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x0000025146AEE470&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000025080972F50&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x0000025080C047D0&gt;)</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.2302956012246557</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0.4211671110684004</v>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>(TerrierRetr(BM25) &gt;&gt; RankCutoff(100) &gt;&gt; &lt;pyterrier.terrier._text_loader.TerrierTextLoader object at 0x0000025081C65CD0&gt; &gt;&gt; (&lt;pyterrier.terrier.retriever.TextScorer object at 0x0000025146AC6750&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000025081867890&gt; ** &lt;pyterrier.terrier.retriever.TextScorer object at 0x0000025081866300&gt; ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score() ** pt.apply.doc_score()) &gt;&gt; &lt;pyterrier.ltr.LTRTransformer object at 0x0000025146986520&gt;)</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.2296936788139386</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0.4172254552213399</v>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>